<commit_message>
Deploying to gh-pages from @ eurovibes/rack-ser-adapter@0b1bb06bfa3c39006344b2b2e95c11755eea03ac 🚀
</commit_message>
<xml_diff>
--- a/Fabrication-tester/BoM/tester-bom_v0.1.xlsx
+++ b/Fabrication-tester/BoM/tester-bom_v0.1.xlsx
@@ -18,33 +18,33 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="189">
   <si>
     <t>Row</t>
   </si>
   <si>
-    <t>Referencias</t>
-  </si>
-  <si>
-    <t>Parte</t>
-  </si>
-  <si>
-    <t>Valor</t>
+    <t>References</t>
+  </si>
+  <si>
+    <t>Part</t>
+  </si>
+  <si>
+    <t>Value</t>
   </si>
   <si>
     <t>P/N</t>
   </si>
   <si>
-    <t>Fabricante</t>
-  </si>
-  <si>
-    <t>Cod. Digi-Key</t>
+    <t>Manufacture</t>
+  </si>
+  <si>
+    <t>Supplier P/N</t>
   </si>
   <si>
     <t>Footprint</t>
   </si>
   <si>
-    <t>Descripción</t>
+    <t>Description</t>
   </si>
   <si>
     <t>Quantity Per PCB</t>
@@ -62,12 +62,21 @@
     <t>10 µF</t>
   </si>
   <si>
+    <t>CL21A106KAYNNNE CL05B104KB54PNC 0402CG200J500NT 0402CG120J500NT CL10A105KB8NNNC</t>
+  </si>
+  <si>
+    <t>Samsung Electro-Mechanics FH (Guangdong Fenghua Advanced Tech)</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
     <t>C_0805_2012Metric</t>
   </si>
   <si>
+    <t>Unpolarized capacitor</t>
+  </si>
+  <si>
     <t>24</t>
   </si>
   <si>
@@ -86,6 +95,9 @@
     <t>CP_Radial_D8.0mm_P3.50mm</t>
   </si>
   <si>
+    <t>Polarized capacitor</t>
+  </si>
+  <si>
     <t>3</t>
   </si>
   <si>
@@ -98,9 +110,15 @@
     <t>1N4148WS</t>
   </si>
   <si>
+    <t>Jiangsu Changjing Electronics Technology Co., Ltd.</t>
+  </si>
+  <si>
     <t>D_SOD-123</t>
   </si>
   <si>
+    <t>75V 0.15A Fast Switching Diode, SOD-123</t>
+  </si>
+  <si>
     <t>4</t>
   </si>
   <si>
@@ -110,9 +128,18 @@
     <t>LED</t>
   </si>
   <si>
+    <t>KT-0603W KT-0603R</t>
+  </si>
+  <si>
+    <t>Hubei KENTO Elec</t>
+  </si>
+  <si>
     <t>LED_0603_1608Metric</t>
   </si>
   <si>
+    <t>Light emitting diode</t>
+  </si>
+  <si>
     <t>34</t>
   </si>
   <si>
@@ -131,6 +158,9 @@
     <t>PinHeader_1x14_P2.54mm_Vertical</t>
   </si>
   <si>
+    <t>Generic connector, single row, 01x14, script generated (kicad-library-utils/schlib/autogen/connector/)</t>
+  </si>
+  <si>
     <t>6</t>
   </si>
   <si>
@@ -146,6 +176,9 @@
     <t>TerminalBlock_WAGO_236-402_1x02_P5.00mm_45Degree</t>
   </si>
   <si>
+    <t>Generic connector, single row, 01x02, script generated (kicad-library-utils/schlib/autogen/connector/)</t>
+  </si>
+  <si>
     <t>7</t>
   </si>
   <si>
@@ -161,6 +194,9 @@
     <t>PinHeader_1x04_P2.54mm_Vertical</t>
   </si>
   <si>
+    <t>Generic connector, single row, 01x04, script generated (kicad-library-utils/schlib/autogen/connector/)</t>
+  </si>
+  <si>
     <t>8</t>
   </si>
   <si>
@@ -170,9 +206,18 @@
     <t>USB_B_Micro</t>
   </si>
   <si>
+    <t>10118194-0001LF</t>
+  </si>
+  <si>
+    <t>Amphenol ICC</t>
+  </si>
+  <si>
     <t>USB_Micro-B_Amphenol_10118193-0001LF_Horizontal</t>
   </si>
   <si>
+    <t>USB Micro Type B connector</t>
+  </si>
+  <si>
     <t>9</t>
   </si>
   <si>
@@ -185,9 +230,18 @@
     <t>X1</t>
   </si>
   <si>
+    <t>DS1037-09MNAKT74-0CC</t>
+  </si>
+  <si>
+    <t>CONNFLY</t>
+  </si>
+  <si>
     <t>DSUB-9_Pins_Vertical_P2.77x2.84mm_MountingHoles</t>
   </si>
   <si>
+    <t>9-pin D-SUB connector, pins (male), Mounting Hole</t>
+  </si>
+  <si>
     <t>10</t>
   </si>
   <si>
@@ -200,9 +254,18 @@
     <t>X2</t>
   </si>
   <si>
+    <t>RJHSE5380</t>
+  </si>
+  <si>
+    <t>AMPHENOL COMMUNICATIONS SOLUTIONS</t>
+  </si>
+  <si>
     <t>RJ45_Amphenol_RJHSE5380</t>
   </si>
   <si>
+    <t>RJ connector, 8P8C (8 positions 8 connected), Shielded</t>
+  </si>
+  <si>
     <t>11</t>
   </si>
   <si>
@@ -215,9 +278,15 @@
     <t>X3</t>
   </si>
   <si>
+    <t>DS1037-09FNAKT74-0CC</t>
+  </si>
+  <si>
     <t>DSUB-9_Socket_Vertical_P2.77x2.84mm_MountingHoles</t>
   </si>
   <si>
+    <t>9-pin D-SUB connector, socket (female), Mounting Hole</t>
+  </si>
+  <si>
     <t>12</t>
   </si>
   <si>
@@ -230,9 +299,15 @@
     <t>SI2301CDS-T1-GE3</t>
   </si>
   <si>
+    <t>Vishay Intertech</t>
+  </si>
+  <si>
     <t>SOT-23</t>
   </si>
   <si>
+    <t>-3A Id, -20V Vds, P-Channel MOSFET, SOT-23</t>
+  </si>
+  <si>
     <t>13</t>
   </si>
   <si>
@@ -245,9 +320,18 @@
     <t>1 kΩ</t>
   </si>
   <si>
+    <t>0402WGF1001TCE 0402WGF4701TCE 0402WGF1002TCE 0402WGF1004TCE 1206W4F220JT5E</t>
+  </si>
+  <si>
+    <t>UNI-ROYAL(Uniroyal Elec)</t>
+  </si>
+  <si>
     <t>R_0402_1005Metric</t>
   </si>
   <si>
+    <t>Resistor</t>
+  </si>
+  <si>
     <t>41</t>
   </si>
   <si>
@@ -263,9 +347,18 @@
     <t>Reset</t>
   </si>
   <si>
+    <t>TACT-65R-F TS-1187A-B-A-B</t>
+  </si>
+  <si>
+    <t>NINIGI XKB Connection</t>
+  </si>
+  <si>
     <t>SW_PUSH_6mm</t>
   </si>
   <si>
+    <t>Push button switch, generic, two pins</t>
+  </si>
+  <si>
     <t>15</t>
   </si>
   <si>
@@ -275,9 +368,15 @@
     <t>AMS1117-3.3</t>
   </si>
   <si>
+    <t>Advanced Monolithic Systems</t>
+  </si>
+  <si>
     <t>SOT-223-3_TabPin2</t>
   </si>
   <si>
+    <t>1A Low Dropout regulator, positive, 3.3V fixed output, SOT-223</t>
+  </si>
+  <si>
     <t>16</t>
   </si>
   <si>
@@ -287,9 +386,15 @@
     <t>CH340N</t>
   </si>
   <si>
+    <t>WCH(Jiangsu Qin Heng)</t>
+  </si>
+  <si>
     <t>JEITA_SOIC-8_3.9x4.9mm_P1.27mm</t>
   </si>
   <si>
+    <t>USB serial converter, 2Mbps, UART, JEITA SOIC-8 (SOP-8)</t>
+  </si>
+  <si>
     <t>17</t>
   </si>
   <si>
@@ -302,9 +407,18 @@
     <t>M24C64-RMN</t>
   </si>
   <si>
+    <t>M24C64-RMN6TP</t>
+  </si>
+  <si>
+    <t>STMicroelectronicsSTMicroelectronics</t>
+  </si>
+  <si>
     <t>SOIC-8_3.9x4.9mm_P1.27mm</t>
   </si>
   <si>
+    <t>2Kb (256x8) I2C Serial EEPROM, 1.8-5.5V, SOIC-8</t>
+  </si>
+  <si>
     <t>18</t>
   </si>
   <si>
@@ -314,9 +428,18 @@
     <t>PCA9539xPW</t>
   </si>
   <si>
+    <t>PCA9539PW</t>
+  </si>
+  <si>
+    <t>NXP Semicon</t>
+  </si>
+  <si>
     <t>TSSOP-24_4.4x7.8mm_P0.65mm</t>
   </si>
   <si>
+    <t>16-bit I/O expander, I2C / SMBus interface, interrupt and reset pins, TSSOP-24</t>
+  </si>
+  <si>
     <t>19</t>
   </si>
   <si>
@@ -326,9 +449,18 @@
     <t>STM32F103C8Tx</t>
   </si>
   <si>
+    <t>STM32F103C8T6</t>
+  </si>
+  <si>
+    <t>STMicroelectronics</t>
+  </si>
+  <si>
     <t>LQFP-48_7x7mm_P0.5mm</t>
   </si>
   <si>
+    <t>STMicroelectronics Arm Cortex-M3 MCU, 64KB flash, 20KB RAM, 72 MHz, 2.0-3.6V, 37 GPIO, LQFP48</t>
+  </si>
+  <si>
     <t>20</t>
   </si>
   <si>
@@ -338,9 +470,15 @@
     <t>USBLC6-2SC6</t>
   </si>
   <si>
+    <t>TECH PUBLIC</t>
+  </si>
+  <si>
     <t>SOT-23-6</t>
   </si>
   <si>
+    <t>Very low capacitance ESD protection diode, 2 data-line, SOT-23-6</t>
+  </si>
+  <si>
     <t>21</t>
   </si>
   <si>
@@ -353,9 +491,18 @@
     <t>XC6206P332MR</t>
   </si>
   <si>
+    <t>XC6206P332MR-G</t>
+  </si>
+  <si>
+    <t>Torex Semicon</t>
+  </si>
+  <si>
     <t>SOT-23-3</t>
   </si>
   <si>
+    <t>Positive 60-250mA Low Dropout Regulator, Fixed Output, SOT-23</t>
+  </si>
+  <si>
     <t>22</t>
   </si>
   <si>
@@ -368,7 +515,16 @@
     <t>8MHz</t>
   </si>
   <si>
+    <t>X50328MSB2GI Q13FC13500004</t>
+  </si>
+  <si>
+    <t>YXC Crystal Oscillators Seiko Epson</t>
+  </si>
+  <si>
     <t>Crystal_SMD_5032-2Pin_5.0x3.2mm</t>
+  </si>
+  <si>
+    <t>Two pin crystal</t>
   </si>
   <si>
     <t>KiBot Bill of Materials</t>
@@ -580,9 +736,9 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>376839</xdr:colOff>
-      <xdr:row>105</xdr:row>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>605439</xdr:colOff>
+      <xdr:row>97</xdr:row>
       <xdr:rowOff>32809</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -914,17 +1070,16 @@
     <col min="2" max="2" width="60.7109375" customWidth="1"/>
     <col min="3" max="3" width="29.7109375" customWidth="1"/>
     <col min="4" max="4" width="52.7109375" customWidth="1"/>
-    <col min="5" max="5" width="19.7109375" customWidth="1"/>
-    <col min="6" max="6" width="20.7109375" customWidth="1"/>
-    <col min="7" max="7" width="23.7109375" customWidth="1"/>
+    <col min="5" max="6" width="60.7109375" customWidth="1"/>
+    <col min="7" max="7" width="22.7109375" customWidth="1"/>
     <col min="8" max="8" width="54.7109375" customWidth="1"/>
-    <col min="9" max="9" width="21.7109375" customWidth="1"/>
+    <col min="9" max="9" width="60.7109375" customWidth="1"/>
     <col min="10" max="10" width="26.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="32" customHeight="1">
       <c r="C1" s="1" t="s">
-        <v>117</v>
+        <v>169</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
@@ -936,13 +1091,13 @@
     </row>
     <row r="2" spans="1:10">
       <c r="C2" s="2" t="s">
-        <v>118</v>
+        <v>170</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>119</v>
+        <v>171</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>128</v>
+        <v>180</v>
       </c>
       <c r="F2" s="3">
         <v>22</v>
@@ -950,13 +1105,13 @@
     </row>
     <row r="3" spans="1:10">
       <c r="C3" s="2" t="s">
-        <v>120</v>
+        <v>172</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>121</v>
+        <v>173</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>129</v>
+        <v>181</v>
       </c>
       <c r="F3" s="3">
         <v>126</v>
@@ -964,13 +1119,13 @@
     </row>
     <row r="4" spans="1:10">
       <c r="C4" s="2" t="s">
-        <v>122</v>
+        <v>174</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>123</v>
+        <v>175</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>130</v>
+        <v>182</v>
       </c>
       <c r="F4" s="3">
         <v>126</v>
@@ -978,13 +1133,13 @@
     </row>
     <row r="5" spans="1:10">
       <c r="C5" s="2" t="s">
-        <v>124</v>
+        <v>176</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>125</v>
+        <v>177</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>131</v>
+        <v>183</v>
       </c>
       <c r="F5" s="3">
         <v>1</v>
@@ -992,13 +1147,13 @@
     </row>
     <row r="6" spans="1:10">
       <c r="C6" s="2" t="s">
-        <v>126</v>
+        <v>178</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>127</v>
+        <v>179</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>132</v>
+        <v>184</v>
       </c>
       <c r="F6" s="3">
         <v>126</v>
@@ -1053,48 +1208,48 @@
         <v>14</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="I9" s="7" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="J9" s="5" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:10">
       <c r="A10" s="8" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F10" s="10" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="J10" s="8" t="s">
         <v>10</v>
@@ -1102,31 +1257,31 @@
     </row>
     <row r="11" spans="1:10">
       <c r="A11" s="5" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="I11" s="7" t="s">
-        <v>14</v>
+        <v>32</v>
       </c>
       <c r="J11" s="5" t="s">
         <v>10</v>
@@ -1134,127 +1289,127 @@
     </row>
     <row r="12" spans="1:10" ht="45" customHeight="1">
       <c r="A12" s="8" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>14</v>
+        <v>36</v>
       </c>
       <c r="F12" s="10" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="J12" s="8" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="30" customHeight="1">
       <c r="A13" s="5" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="I13" s="7" t="s">
-        <v>14</v>
+        <v>46</v>
       </c>
       <c r="J13" s="5" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:10">
+    <row r="14" spans="1:10" ht="30" customHeight="1">
       <c r="A14" s="8" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F14" s="10" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>14</v>
+        <v>52</v>
       </c>
       <c r="J14" s="8" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:10">
+    <row r="15" spans="1:10" ht="30" customHeight="1">
       <c r="A15" s="5" t="s">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>45</v>
+        <v>56</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>46</v>
+        <v>57</v>
       </c>
       <c r="I15" s="7" t="s">
-        <v>14</v>
+        <v>58</v>
       </c>
       <c r="J15" s="5" t="s">
         <v>10</v>
@@ -1262,31 +1417,31 @@
     </row>
     <row r="16" spans="1:10">
       <c r="A16" s="8" t="s">
-        <v>47</v>
+        <v>59</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>49</v>
+        <v>61</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>49</v>
+        <v>61</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>14</v>
+        <v>62</v>
       </c>
       <c r="F16" s="10" t="s">
-        <v>14</v>
+        <v>63</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>50</v>
+        <v>64</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>14</v>
+        <v>65</v>
       </c>
       <c r="J16" s="8" t="s">
         <v>10</v>
@@ -1294,31 +1449,31 @@
     </row>
     <row r="17" spans="1:10">
       <c r="A17" s="5" t="s">
-        <v>51</v>
+        <v>66</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>53</v>
+        <v>68</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>54</v>
+        <v>69</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>14</v>
+        <v>70</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>14</v>
+        <v>71</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>55</v>
+        <v>72</v>
       </c>
       <c r="I17" s="7" t="s">
-        <v>14</v>
+        <v>73</v>
       </c>
       <c r="J17" s="5" t="s">
         <v>10</v>
@@ -1326,31 +1481,31 @@
     </row>
     <row r="18" spans="1:10">
       <c r="A18" s="8" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>59</v>
+        <v>77</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>14</v>
+        <v>78</v>
       </c>
       <c r="F18" s="10" t="s">
-        <v>14</v>
+        <v>79</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>14</v>
+        <v>81</v>
       </c>
       <c r="J18" s="8" t="s">
         <v>10</v>
@@ -1358,31 +1513,31 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" s="5" t="s">
-        <v>61</v>
+        <v>82</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>62</v>
+        <v>83</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>63</v>
+        <v>84</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>64</v>
+        <v>85</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>14</v>
+        <v>86</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>14</v>
+        <v>71</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>65</v>
+        <v>87</v>
       </c>
       <c r="I19" s="7" t="s">
-        <v>14</v>
+        <v>88</v>
       </c>
       <c r="J19" s="5" t="s">
         <v>10</v>
@@ -1390,31 +1545,31 @@
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="8" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>68</v>
+        <v>91</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>69</v>
+        <v>92</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>14</v>
+        <v>92</v>
       </c>
       <c r="F20" s="10" t="s">
-        <v>14</v>
+        <v>93</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>70</v>
+        <v>94</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>14</v>
+        <v>95</v>
       </c>
       <c r="J20" s="8" t="s">
         <v>10</v>
@@ -1422,95 +1577,95 @@
     </row>
     <row r="21" spans="1:10" ht="60" customHeight="1">
       <c r="A21" s="5" t="s">
-        <v>71</v>
+        <v>96</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>72</v>
+        <v>97</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>73</v>
+        <v>98</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>74</v>
+        <v>99</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>14</v>
+        <v>100</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>14</v>
+        <v>101</v>
       </c>
       <c r="G21" s="7" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>75</v>
+        <v>102</v>
       </c>
       <c r="I21" s="7" t="s">
-        <v>14</v>
+        <v>103</v>
       </c>
       <c r="J21" s="5" t="s">
-        <v>76</v>
+        <v>104</v>
       </c>
     </row>
     <row r="22" spans="1:10">
       <c r="A22" s="8" t="s">
-        <v>77</v>
+        <v>105</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>78</v>
+        <v>106</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>79</v>
+        <v>107</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>80</v>
+        <v>108</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>14</v>
+        <v>109</v>
       </c>
       <c r="F22" s="10" t="s">
-        <v>14</v>
+        <v>110</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>81</v>
+        <v>111</v>
       </c>
       <c r="I22" s="10" t="s">
-        <v>14</v>
+        <v>112</v>
       </c>
       <c r="J22" s="8" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="30" customHeight="1">
       <c r="A23" s="5" t="s">
-        <v>82</v>
+        <v>113</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>83</v>
+        <v>114</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>84</v>
+        <v>115</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>84</v>
+        <v>115</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>14</v>
+        <v>115</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>14</v>
+        <v>116</v>
       </c>
       <c r="G23" s="7" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H23" s="6" t="s">
-        <v>85</v>
+        <v>117</v>
       </c>
       <c r="I23" s="7" t="s">
-        <v>14</v>
+        <v>118</v>
       </c>
       <c r="J23" s="5" t="s">
         <v>10</v>
@@ -1518,31 +1673,31 @@
     </row>
     <row r="24" spans="1:10">
       <c r="A24" s="8" t="s">
-        <v>86</v>
+        <v>119</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>87</v>
+        <v>120</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>88</v>
+        <v>121</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>88</v>
+        <v>121</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>14</v>
+        <v>121</v>
       </c>
       <c r="F24" s="10" t="s">
-        <v>14</v>
+        <v>122</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>89</v>
+        <v>123</v>
       </c>
       <c r="I24" s="10" t="s">
-        <v>14</v>
+        <v>124</v>
       </c>
       <c r="J24" s="8" t="s">
         <v>10</v>
@@ -1550,159 +1705,159 @@
     </row>
     <row r="25" spans="1:10">
       <c r="A25" s="5" t="s">
-        <v>90</v>
+        <v>125</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>91</v>
+        <v>126</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>92</v>
+        <v>127</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>93</v>
+        <v>128</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>14</v>
+        <v>129</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>14</v>
+        <v>130</v>
       </c>
       <c r="G25" s="7" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H25" s="6" t="s">
-        <v>94</v>
+        <v>131</v>
       </c>
       <c r="I25" s="7" t="s">
-        <v>14</v>
+        <v>132</v>
       </c>
       <c r="J25" s="5" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="30" customHeight="1">
       <c r="A26" s="8" t="s">
-        <v>95</v>
+        <v>133</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>96</v>
+        <v>134</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>97</v>
+        <v>135</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>97</v>
+        <v>135</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>14</v>
+        <v>136</v>
       </c>
       <c r="F26" s="10" t="s">
-        <v>14</v>
+        <v>137</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>98</v>
+        <v>138</v>
       </c>
       <c r="I26" s="10" t="s">
-        <v>14</v>
+        <v>139</v>
       </c>
       <c r="J26" s="8" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="30" customHeight="1">
       <c r="A27" s="5" t="s">
-        <v>99</v>
+        <v>140</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>100</v>
+        <v>141</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>101</v>
+        <v>142</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>101</v>
+        <v>142</v>
       </c>
       <c r="E27" s="7" t="s">
-        <v>14</v>
+        <v>143</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>14</v>
+        <v>144</v>
       </c>
       <c r="G27" s="7" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H27" s="6" t="s">
-        <v>102</v>
+        <v>145</v>
       </c>
       <c r="I27" s="7" t="s">
-        <v>14</v>
+        <v>146</v>
       </c>
       <c r="J27" s="5" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="28" spans="1:10">
+    <row r="28" spans="1:10" ht="30" customHeight="1">
       <c r="A28" s="8" t="s">
-        <v>103</v>
+        <v>147</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>104</v>
+        <v>148</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>105</v>
+        <v>149</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>105</v>
+        <v>149</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>14</v>
+        <v>149</v>
       </c>
       <c r="F28" s="10" t="s">
-        <v>14</v>
+        <v>150</v>
       </c>
       <c r="G28" s="10" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>106</v>
+        <v>151</v>
       </c>
       <c r="I28" s="10" t="s">
-        <v>14</v>
+        <v>152</v>
       </c>
       <c r="J28" s="8" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="29" spans="1:10">
+    <row r="29" spans="1:10" ht="30" customHeight="1">
       <c r="A29" s="5" t="s">
-        <v>107</v>
+        <v>153</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>108</v>
+        <v>154</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>109</v>
+        <v>155</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>110</v>
+        <v>156</v>
       </c>
       <c r="E29" s="7" t="s">
-        <v>14</v>
+        <v>157</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>14</v>
+        <v>158</v>
       </c>
       <c r="G29" s="7" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H29" s="6" t="s">
-        <v>111</v>
+        <v>159</v>
       </c>
       <c r="I29" s="7" t="s">
-        <v>14</v>
+        <v>160</v>
       </c>
       <c r="J29" s="5" t="s">
         <v>10</v>
@@ -1710,34 +1865,34 @@
     </row>
     <row r="30" spans="1:10">
       <c r="A30" s="8" t="s">
-        <v>112</v>
+        <v>161</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>113</v>
+        <v>162</v>
       </c>
       <c r="C30" s="9" t="s">
-        <v>114</v>
+        <v>163</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>115</v>
+        <v>164</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>14</v>
+        <v>165</v>
       </c>
       <c r="F30" s="10" t="s">
-        <v>14</v>
+        <v>166</v>
       </c>
       <c r="G30" s="10" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>116</v>
+        <v>167</v>
       </c>
       <c r="I30" s="10" t="s">
-        <v>14</v>
+        <v>168</v>
       </c>
       <c r="J30" s="8" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -1784,22 +1939,22 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>133</v>
+        <v>185</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="6" t="s">
-        <v>134</v>
+        <v>186</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="5" t="s">
-        <v>135</v>
+        <v>187</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="7" t="s">
-        <v>136</v>
+        <v>188</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ eurovibes/rack-ser-adapter@b037410175b53bc71bd1758dfd46abdfa03946e2 🚀
</commit_message>
<xml_diff>
--- a/Fabrication-tester/BoM/tester-bom_v0.1.xlsx
+++ b/Fabrication-tester/BoM/tester-bom_v0.1.xlsx
@@ -110,10 +110,10 @@
     <t>1N4148WS</t>
   </si>
   <si>
-    <t>Jiangsu Changjing Electronics Technology Co., Ltd.</t>
-  </si>
-  <si>
-    <t>D_SOD-323</t>
+    <t>ST(Semtech)</t>
+  </si>
+  <si>
+    <t>D_SOD-123</t>
   </si>
   <si>
     <t>75V 0.15A Fast Switching Diode, SOD-123</t>
@@ -1269,7 +1269,7 @@
         <v>29</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F11" s="7" t="s">
         <v>30</v>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ eurovibes/rack-ser-adapter@b8f255b1baa0435bdff679e7bcf8e275f3efaa27 🚀
</commit_message>
<xml_diff>
--- a/Fabrication-tester/BoM/tester-bom_v0.1.xlsx
+++ b/Fabrication-tester/BoM/tester-bom_v0.1.xlsx
@@ -206,7 +206,7 @@
     <t>USB_B_Micro</t>
   </si>
   <si>
-    <t>10118194-0001LF</t>
+    <t>10118193-0001LF</t>
   </si>
   <si>
     <t>Amphenol ICC</t>
@@ -248,7 +248,7 @@
     <t>J103</t>
   </si>
   <si>
-    <t>RJ45_Shielded</t>
+    <t>RJ45_LED_Shielded</t>
   </si>
   <si>
     <t>X2</t>
@@ -260,10 +260,10 @@
     <t>AMPHENOL COMMUNICATIONS SOLUTIONS</t>
   </si>
   <si>
-    <t>RJ45_Amphenol_RJHSE5380</t>
-  </si>
-  <si>
-    <t>RJ connector, 8P8C (8 positions 8 connected), Shielded</t>
+    <t>RJ45_Amphenol_RJHSE538X</t>
+  </si>
+  <si>
+    <t>RJ connector, 8P8C (8 positions 8 connected), two LEDs, Shielded</t>
   </si>
   <si>
     <t>11</t>
@@ -311,7 +311,7 @@
     <t>13</t>
   </si>
   <si>
-    <t>R101 R102 R103 R104 R105 R106 R107 R108 R109 R110 R111 R112 R113 R114 R115 R116 R117 R118 R119 R120 R121 R122 R123 R124 R125 R126 R127 R128 R129 R130 R131 R132 R133 R134 R201 R202 R203 R204 R205 R206 R401</t>
+    <t>R101 R102 R103 R104 R105 R106 R107 R108 R109 R110 R111 R112 R113 R114 R115 R116 R117 R118 R119 R120 R121 R122 R123 R124 R125 R126 R127 R128 R129 R130 R131 R132 R133 R134 R135 R136 R201 R202 R203 R204 R205 R206 R207 R208 R401</t>
   </si>
   <si>
     <t>R</t>
@@ -332,7 +332,7 @@
     <t>Resistor</t>
   </si>
   <si>
-    <t>41</t>
+    <t>45</t>
   </si>
   <si>
     <t>14</t>
@@ -738,7 +738,7 @@
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>605439</xdr:colOff>
-      <xdr:row>97</xdr:row>
+      <xdr:row>96</xdr:row>
       <xdr:rowOff>32809</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1114,7 +1114,7 @@
         <v>181</v>
       </c>
       <c r="F3" s="3">
-        <v>126</v>
+        <v>130</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -1128,7 +1128,7 @@
         <v>182</v>
       </c>
       <c r="F4" s="3">
-        <v>126</v>
+        <v>130</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -1156,7 +1156,7 @@
         <v>184</v>
       </c>
       <c r="F6" s="3">
-        <v>126</v>
+        <v>130</v>
       </c>
     </row>
     <row r="8" spans="1:10">
@@ -1479,7 +1479,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="1:10">
+    <row r="18" spans="1:10" ht="30" customHeight="1">
       <c r="A18" s="8" t="s">
         <v>74</v>
       </c>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ eurovibes/rack-ser-adapter@d95818e18515b2a3e123096b8cd82a0300ad2269 🚀
</commit_message>
<xml_diff>
--- a/Fabrication-tester/BoM/tester-bom_v0.1.xlsx
+++ b/Fabrication-tester/BoM/tester-bom_v0.1.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="191">
   <si>
     <t>Row</t>
   </si>
@@ -83,16 +83,22 @@
     <t>2</t>
   </si>
   <si>
-    <t>C212</t>
+    <t>C209 C212</t>
   </si>
   <si>
     <t>C_Polarized</t>
   </si>
   <si>
-    <t>1 F</t>
-  </si>
-  <si>
-    <t>CP_Radial_D8.0mm_P3.50mm</t>
+    <t>22 µF</t>
+  </si>
+  <si>
+    <t>CA45-A-10V-22uF-K</t>
+  </si>
+  <si>
+    <t>CEC(Shenzhen Zhenhua XinYun Elec)</t>
+  </si>
+  <si>
+    <t>C_1206_3216Metric</t>
   </si>
   <si>
     <t>Polarized capacitor</t>
@@ -1079,7 +1085,7 @@
   <sheetData>
     <row r="1" spans="1:10" ht="32" customHeight="1">
       <c r="C1" s="1" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
@@ -1091,13 +1097,13 @@
     </row>
     <row r="2" spans="1:10">
       <c r="C2" s="2" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="F2" s="3">
         <v>22</v>
@@ -1105,41 +1111,41 @@
     </row>
     <row r="3" spans="1:10">
       <c r="C3" s="2" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="F3" s="3">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="4" spans="1:10">
       <c r="C4" s="2" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="F4" s="3">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="5" spans="1:10">
       <c r="C5" s="2" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="F5" s="3">
         <v>1</v>
@@ -1147,16 +1153,16 @@
     </row>
     <row r="6" spans="1:10">
       <c r="C6" s="2" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="F6" s="3">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="8" spans="1:10">
@@ -1237,51 +1243,51 @@
         <v>23</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="F10" s="10" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="G10" s="10" t="s">
         <v>16</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="J10" s="8" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:10">
       <c r="A11" s="5" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="G11" s="7" t="s">
         <v>16</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="I11" s="7" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="J11" s="5" t="s">
         <v>10</v>
@@ -1289,48 +1295,48 @@
     </row>
     <row r="12" spans="1:10" ht="45" customHeight="1">
       <c r="A12" s="8" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F12" s="10" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G12" s="10" t="s">
         <v>16</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="J12" s="8" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="30" customHeight="1">
       <c r="A13" s="5" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E13" s="7" t="s">
         <v>16</v>
@@ -1342,10 +1348,10 @@
         <v>16</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="I13" s="7" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="J13" s="5" t="s">
         <v>10</v>
@@ -1353,16 +1359,16 @@
     </row>
     <row r="14" spans="1:10" ht="30" customHeight="1">
       <c r="A14" s="8" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E14" s="10" t="s">
         <v>16</v>
@@ -1374,10 +1380,10 @@
         <v>16</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="J14" s="8" t="s">
         <v>10</v>
@@ -1385,16 +1391,16 @@
     </row>
     <row r="15" spans="1:10" ht="30" customHeight="1">
       <c r="A15" s="5" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E15" s="7" t="s">
         <v>16</v>
@@ -1406,10 +1412,10 @@
         <v>16</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="I15" s="7" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="J15" s="5" t="s">
         <v>10</v>
@@ -1417,31 +1423,31 @@
     </row>
     <row r="16" spans="1:10">
       <c r="A16" s="8" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F16" s="10" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="G16" s="10" t="s">
         <v>16</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="J16" s="8" t="s">
         <v>10</v>
@@ -1449,31 +1455,31 @@
     </row>
     <row r="17" spans="1:10">
       <c r="A17" s="5" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="G17" s="7" t="s">
         <v>16</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I17" s="7" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="J17" s="5" t="s">
         <v>10</v>
@@ -1481,31 +1487,31 @@
     </row>
     <row r="18" spans="1:10" ht="30" customHeight="1">
       <c r="A18" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="F18" s="10" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="G18" s="10" t="s">
         <v>16</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="J18" s="8" t="s">
         <v>10</v>
@@ -1513,31 +1519,31 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" s="5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="G19" s="7" t="s">
         <v>16</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="I19" s="7" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="J19" s="5" t="s">
         <v>10</v>
@@ -1545,31 +1551,31 @@
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="8" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="F20" s="10" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="G20" s="10" t="s">
         <v>16</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="J20" s="8" t="s">
         <v>10</v>
@@ -1577,95 +1583,95 @@
     </row>
     <row r="21" spans="1:10" ht="60" customHeight="1">
       <c r="A21" s="5" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="G21" s="7" t="s">
         <v>16</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="I21" s="7" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="J21" s="5" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="22" spans="1:10">
       <c r="A22" s="8" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="F22" s="10" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="G22" s="10" t="s">
         <v>16</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="I22" s="10" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="J22" s="8" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="23" spans="1:10" ht="30" customHeight="1">
       <c r="A23" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="G23" s="7" t="s">
         <v>16</v>
       </c>
       <c r="H23" s="6" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="I23" s="7" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="J23" s="5" t="s">
         <v>10</v>
@@ -1673,31 +1679,31 @@
     </row>
     <row r="24" spans="1:10">
       <c r="A24" s="8" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F24" s="10" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>16</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="I24" s="10" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="J24" s="8" t="s">
         <v>10</v>
@@ -1705,31 +1711,31 @@
     </row>
     <row r="25" spans="1:10">
       <c r="A25" s="5" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="G25" s="7" t="s">
         <v>16</v>
       </c>
       <c r="H25" s="6" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="I25" s="7" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="J25" s="5" t="s">
         <v>20</v>
@@ -1737,31 +1743,31 @@
     </row>
     <row r="26" spans="1:10" ht="30" customHeight="1">
       <c r="A26" s="8" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F26" s="10" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>16</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="I26" s="10" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="J26" s="8" t="s">
         <v>20</v>
@@ -1769,31 +1775,31 @@
     </row>
     <row r="27" spans="1:10" ht="30" customHeight="1">
       <c r="A27" s="5" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="E27" s="7" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="G27" s="7" t="s">
         <v>16</v>
       </c>
       <c r="H27" s="6" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="I27" s="7" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="J27" s="5" t="s">
         <v>10</v>
@@ -1801,31 +1807,31 @@
     </row>
     <row r="28" spans="1:10" ht="30" customHeight="1">
       <c r="A28" s="8" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="F28" s="10" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="G28" s="10" t="s">
         <v>16</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="I28" s="10" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="J28" s="8" t="s">
         <v>10</v>
@@ -1833,31 +1839,31 @@
     </row>
     <row r="29" spans="1:10" ht="30" customHeight="1">
       <c r="A29" s="5" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="E29" s="7" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="G29" s="7" t="s">
         <v>16</v>
       </c>
       <c r="H29" s="6" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="I29" s="7" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="J29" s="5" t="s">
         <v>10</v>
@@ -1865,31 +1871,31 @@
     </row>
     <row r="30" spans="1:10">
       <c r="A30" s="8" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C30" s="9" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="F30" s="10" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="G30" s="10" t="s">
         <v>16</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="I30" s="10" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="J30" s="8" t="s">
         <v>20</v>
@@ -1939,22 +1945,22 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="6" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="5" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="7" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
     </row>
   </sheetData>

</xml_diff>